<commit_message>
Update layout parameters and modify analysis files
- Adjusted linkDistance and repelForce in quartz.layout.ts for improved layout dynamics.
- Updated multiple Excel files in the vault-dalarna-university repository, reflecting changes in grading scales, Bloom taxonomy, examination formats, and consistency in phrasing.
- Revised markdown files to reflect the correct number of entries and updated download links for the corresponding Excel files.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AFT2C8</t>
+          <t>AFT2CA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -487,19 +487,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>`generalizability` (en)</t>
+          <t>`framworks` (en)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2CA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AFT2C8</t>
+          <t>AFT2CA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -514,24 +514,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>`transferability` (en)</t>
+          <t>`scienfific` (en)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2CA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AFT2CA</t>
+          <t>AIH237</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FYS</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -541,24 +541,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>`framworks` (en)</t>
+          <t>`cedits` (en)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2CA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIH237</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AFT2CA</t>
+          <t>GIH2D5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FYS</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -568,19 +568,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>`scienfific` (en)</t>
+          <t>`individualising` (en)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2CA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2D5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AIH237</t>
+          <t>GIH2DB</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -590,24 +590,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>`cedits` (en)</t>
+          <t>`jämviktsystem` → jämviktssystem</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIH237</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2DB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GIH2D5</t>
+          <t>GIH2DB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -617,24 +617,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>`focussing` (en)</t>
+          <t>`jämviktsystem` (sv)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2DB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GIH2D5</t>
+          <t>GIH2DC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -644,24 +644,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>`fulfilment` (en)</t>
+          <t>`jämviktsystem` → jämviktssystem</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2DC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GIH2D5</t>
+          <t>GIH2DC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -671,24 +671,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>`individualisation` (en)</t>
+          <t>`jämviktsystem` (sv)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2DC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GIH2D5</t>
+          <t>GIH2NR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -703,19 +703,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>`individualising` (en)</t>
+          <t>`lecturs` (en)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2NR</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GIH2DB</t>
+          <t>GIH2QL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -730,19 +730,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>`jämviktsystem` (sv)</t>
+          <t>`idrottsränarprogrammet` (sv)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2DB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GIH2DC</t>
+          <t>GIH2WX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -757,19 +757,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>`jämviktsystem` (sv)</t>
+          <t>`lärar` (sv)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2DC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WX</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GIH2NR</t>
+          <t>GIH2ZA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>`lecturs` (en)</t>
+          <t>`enviroment` (en)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2NR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GIH2NR</t>
+          <t>GIH2ZB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -806,24 +806,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>`sensorimotor` (en)</t>
+          <t>`idrottsläramoment` (sv)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2NR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GIH2QK</t>
+          <t>GIH2ZC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -833,24 +833,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>`testläraprinciper` (sv)</t>
+          <t>`movementorgans` (en)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GIH2QL</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -860,24 +860,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>`idrottsränarprogrammet` (sv)</t>
+          <t>`asignment` (en)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GIH2WX</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>`lärar` (sv)</t>
+          <t>`asignments` (en)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZA</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>`enviroment` (en)</t>
+          <t>`collaboratation` (en)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZB</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -941,24 +941,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>`idrottsläramoment` (sv)</t>
+          <t>`reciece` (en)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZC</t>
+          <t>GIH335</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -968,24 +968,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>`movementorgans` (en)</t>
+          <t>`soloprenör` (sv)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH335</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GIH33P</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -995,24 +995,24 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>`asignment` (en)</t>
+          <t>`jämviktsystem` → jämviktssystem</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GIH33P</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1022,24 +1022,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>`asignments` (en)</t>
+          <t>`jämviktsystem` (sv)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GIH34D</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1054,19 +1054,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>`collaboratation` (en)</t>
+          <t>`humanistiv` (en)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GIH34T</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1081,19 +1081,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>`reciece` (en)</t>
+          <t>`respirationsystem` (en)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GIH335</t>
+          <t>GIH37S</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1103,24 +1103,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>`soloprenör` (sv)</t>
+          <t>`enviroment` (en)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH335</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37S</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GIH33P</t>
+          <t>GIH38Y</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1130,24 +1130,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>`jämviktsystem` (sv)</t>
+          <t>`respirationsystem` (en)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH38Y</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GIH34D</t>
+          <t>GIH393</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1157,24 +1157,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`humanistiv` (en)</t>
+          <t>`idrottsläramoment` (sv)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH393</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GIH34T</t>
+          <t>GIH394</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1184,24 +1184,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`respirationsystem` (en)</t>
+          <t>`lärar` (sv)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH394</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GIH37S</t>
+          <t>GIH39D</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1221,14 +1221,14 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH39D</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GIH38Y</t>
+          <t>GIH39H</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1243,19 +1243,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`respirationsystem` (en)</t>
+          <t>`movementorgans` (en)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH38Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH39H</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GIH393</t>
+          <t>GIH3AQ</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1270,19 +1270,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>`idrottsläramoment` (sv)</t>
+          <t>`mätprinciper` (sv)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH393</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GIH394</t>
+          <t>GIH3C2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1292,24 +1292,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>`lärar` (sv)</t>
+          <t>`reporage` (en)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH394</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3C2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GIH39D</t>
+          <t>GIH3D5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1319,24 +1319,24 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>`enviroment` (en)</t>
+          <t>`hälsopromotiva` (sv)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH39D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GIH39H</t>
+          <t>GIH3F7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1346,24 +1346,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>`movementorgans` (en)</t>
+          <t>`normförmedlare` (sv)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH39H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F7</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GIH3AQ</t>
+          <t>GIH3F7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1373,24 +1373,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>`mätprinciper` (sv)</t>
+          <t>`teories` (en)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F7</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GIH3C2</t>
+          <t>GIH3G6</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1400,24 +1400,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>`reporage` (en)</t>
+          <t>`kunskapnivå` (sv)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3C2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GIH3D5</t>
+          <t>GIH3G8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1427,24 +1427,24 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>`hälsopromotiva` (sv)</t>
+          <t>`intrapersonal` (en)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GIH3F7</t>
+          <t>GIH3G9</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1459,19 +1459,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>`normförmedlare` (sv)</t>
+          <t>`soloprenör` (sv)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GIH3F7</t>
+          <t>GIH3G9</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1486,19 +1486,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>`teories` (en)</t>
+          <t>`intrapreneur` (en)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GIH3G6</t>
+          <t>GIH3G9</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1508,24 +1508,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>`kunskapnivå` (sv)</t>
+          <t>`solopreneur` (en)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GIH3G8</t>
+          <t>GIH3JL</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1540,19 +1540,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>`intrapersonal` (en)</t>
+          <t>`emphasising` (en)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GIH3G9</t>
+          <t>IH1001</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1567,19 +1567,19 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>`soloprenör` (sv)</t>
+          <t>`rörel-sekompetensen` (sv)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1001</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GIH3G9</t>
+          <t>IH1003</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1594,19 +1594,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>`intrapreneur` (en)</t>
+          <t>`leasure` (en)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GIH3G9</t>
+          <t>IH1003</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1621,19 +1621,19 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>`solopreneur` (en)</t>
+          <t>`workingform` (en)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GIH3JL</t>
+          <t>IH1004</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1648,19 +1648,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>`emphasising` (en)</t>
+          <t>`peda` (en)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1004</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>IH1001</t>
+          <t>IH1024</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1675,19 +1675,19 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>`rörel-sekompetensen` (sv)</t>
+          <t>`förläsningar` (sv)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1024</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>IH1003</t>
+          <t>IH1062</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1697,24 +1697,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>`leasure` (en)</t>
+          <t>`kärlproblematik` (sv)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1062</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>IH1003</t>
+          <t>IH1062</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>`workingform` (en)</t>
+          <t>`vätske` (sv)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1062</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IH1004</t>
+          <t>IH1114</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1751,24 +1751,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>`peda` (en)</t>
+          <t>`hjäipmedels` (sv)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1114</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>IH1024</t>
+          <t>IH1122</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1778,24 +1778,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>`förläsningar` (sv)</t>
+          <t>`hisory` (en)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1122</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>IH1062</t>
+          <t>IH2002</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1805,24 +1805,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>`kärlproblematik` (sv)</t>
+          <t>`rythm` (en)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1062</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2002</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>IH1062</t>
+          <t>IH3007</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1832,24 +1832,24 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>`vätske` (sv)</t>
+          <t>`humanbiologi` (en)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1062</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH3007</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>IH1114</t>
+          <t>IH3007</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1859,56 +1859,56 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>`hjäipmedels` (sv)</t>
+          <t>`idrottsinriktning` (en)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1114</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH3007</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>IH1122</t>
+          <t>BKE223</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>KEA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>`hisory` (en)</t>
+          <t>`stökiometri` (sv)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1122</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>IH1130</t>
+          <t>BKE223</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>KEA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1918,24 +1918,24 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>`testläraprinciper` (sv)</t>
+          <t>`substansmängdsförhållanden` (sv)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1130</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>IH2002</t>
+          <t>AMC243</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1945,24 +1945,24 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>`rythm` (en)</t>
+          <t>`naprapath` (en)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>IH3007</t>
+          <t>AMC243</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1972,51 +1972,51 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>`humanbiologi` (en)</t>
+          <t>`physiotherpy` (en)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>IH3007</t>
+          <t>AMC25W</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>`idrottsinriktning` (en)</t>
+          <t>`ehälsa` (sv)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC25W</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>BKE223</t>
+          <t>AMC265</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>KEA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2026,46 +2026,46 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>`stökiometri` (sv)</t>
+          <t>`sjuksköterske` (sv)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC265</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>BKE223</t>
+          <t>AMC265</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KEA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>`substansmängdsförhållanden` (sv)</t>
+          <t>`dietician` (en)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC265</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>AMC2A7</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2080,19 +2080,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>`naprapath` (en)</t>
+          <t>`arrhythmias` (en)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>GMC2AH</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2102,24 +2102,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>`physiotherpy` (en)</t>
+          <t>`vätske` (sv)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMC2AH</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AMC25W</t>
+          <t>MC2023</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2134,78 +2134,78 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>`ehälsa` (sv)</t>
+          <t>`kärlområdet` (sv)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC25W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MC2023</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AMC265</t>
+          <t>GNV396</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>`sjuksköterske` (sv)</t>
+          <t>`artefacts` (en)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC265</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AMC265</t>
+          <t>GNV3GU</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>`dietician` (en)</t>
+          <t>`inlämingsuppgift` (sv)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC265</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AMC2A7</t>
+          <t>GNV3GU</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2215,24 +2215,24 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>`arrhythmias` (en)</t>
+          <t>`natur` (en)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GMC2AH</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2242,46 +2242,46 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>`vätske` (sv)</t>
+          <t>`inlämingsuppgift` (sv)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMC2AH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>MC2023</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>`kärlområdet` (sv)</t>
+          <t>`historia` (en)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MC2023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GNV396</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2296,19 +2296,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>`artefacts` (en)</t>
+          <t>`naturvetenskap` (en)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GNV3GU</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2318,24 +2318,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>`inlämingsuppgift` (sv)</t>
+          <t>`naturvetenskapernas` (en)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GNV3GU</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>`natur` (en)</t>
+          <t>`naturvetenskapliga` (en)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
@@ -2372,12 +2372,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>`inlämingsuppgift` (sv)</t>
+          <t>`vardag` (en)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2389,7 +2389,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>NV1024</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>`historia` (en)</t>
+          <t>`educationas` (en)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1024</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>NV1027</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>`naturvetenskap` (en)</t>
+          <t>`adresses` (en)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1027</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>NV3001</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2453,29 +2453,29 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>`naturvetenskapernas` (en)</t>
+          <t>`förståelser` (sv)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV3001</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>ASA24N</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2485,24 +2485,24 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>`naturvetenskapliga` (en)</t>
+          <t>`engelskt` (en)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA24N</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>ASA24N</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2512,24 +2512,24 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>`vardag` (en)</t>
+          <t>`namn` (en)</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA24N</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>NV1024</t>
+          <t>ASA28Q</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2539,73 +2539,73 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>`educationas` (en)</t>
+          <t>`researcg` (en)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA28Q</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>NV1027</t>
+          <t>GSA2NC</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>`adresses` (en)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>NV3001</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>`förståelser` (sv)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV3001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ASA24N</t>
+          <t>GSA352</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2620,19 +2620,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>`engelskt` (en)</t>
+          <t>`assignmentss` (en)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA24N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA352</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>ASA24N</t>
+          <t>GSA3AS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2647,19 +2647,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>`namn` (en)</t>
+          <t>`interorganizational` (en)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA24N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ASA28Q</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2669,24 +2669,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>`researcg` (en)</t>
+          <t>`brukarperspektivinnebär` (sv)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA28Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GSA2NC</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2696,24 +2696,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
+          <t>`frånorganisationsperspektiv` (sv)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2723,24 +2723,24 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
+          <t>`somarbetslöshet` (sv)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>GSA352</t>
+          <t>GSA3DN</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>`assignmentss` (en)</t>
+          <t>`sem` (en)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA352</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>GSA3DP</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2782,19 +2782,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>`interorganizational` (en)</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>SA1037</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2809,19 +2809,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>`brukarperspektivinnebär` (sv)</t>
+          <t>`övergripandemål` (sv)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1037</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2836,19 +2836,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>`frånorganisationsperspektiv` (sv)</t>
+          <t>`självtillitsträning` (sv)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2863,19 +2863,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>`somarbetslöshet` (sv)</t>
+          <t>`skalfrågor` (sv)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>GSA3DN</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2885,24 +2885,24 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>`sem` (en)</t>
+          <t>`utvärderbara` (sv)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>GSA3DP</t>
+          <t>SA2020</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2912,110 +2912,110 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>`guidlines` (en)</t>
+          <t>`fördjuping` (sv)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>SA1037</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>`övergripandemål` (sv)</t>
+          <t>`ethhtical` (en)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1037</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>`självtillitsträning` (sv)</t>
+          <t>`summarisze` (en)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR25V</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>`skalfrågor` (sv)</t>
+          <t>`systemacity` (en)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR26N</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3025,24 +3025,24 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>`utvärderbara` (sv)</t>
+          <t>`läraktivitet` (sv)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>ASR26N</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3052,19 +3052,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>`fördjuping` (sv)</t>
+          <t>`läraktiviteter` (sv)</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3079,19 +3079,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>`ethhtical` (en)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3106,19 +3106,19 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>`summarisze` (en)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ASR25V</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3133,19 +3133,19 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>`systemacity` (en)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ASR26N</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3155,24 +3155,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>`läraktivitet` (sv)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>ASR26N</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3182,24 +3182,24 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>`läraktiviteter` (sv)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3214,19 +3214,19 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3241,19 +3241,19 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`alsoincludes` (en)</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3268,19 +3268,19 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`anotherstudent` (en)</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3295,19 +3295,19 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`compilinga` (en)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3322,19 +3322,19 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`thesisand` (en)</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3344,24 +3344,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`föräldrablivande` (sv)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3376,19 +3376,19 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>`alsoincludes` (en)</t>
+          <t>`beable` (en)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3403,19 +3403,19 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>`anotherstudent` (en)</t>
+          <t>`processesof` (en)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3430,19 +3430,19 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>`compilinga` (en)</t>
+          <t>`thestudent` (en)</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3457,19 +3457,19 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>`thesisand` (en)</t>
+          <t>`toconduct` (en)</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3479,24 +3479,24 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>`föräldrablivande` (sv)</t>
+          <t>`ofthe` (en)</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3511,19 +3511,19 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>`beable` (en)</t>
+          <t>`postpartumperiod` (en)</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3538,19 +3538,19 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>`processesof` (en)</t>
+          <t>`srole` (en)</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3565,19 +3565,19 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>`thestudent` (en)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3592,19 +3592,19 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>`toconduct` (en)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3619,19 +3619,19 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>`ofthe` (en)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3646,19 +3646,19 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>`postpartumperiod` (en)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3673,19 +3673,19 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>`srole` (en)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR29W</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3700,19 +3700,19 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3722,24 +3722,24 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`förforskningsområdet` (sv)</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3749,24 +3749,24 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`reproduktivhälsaoch` (sv)</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CH</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3781,19 +3781,19 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`perspectiv` (en)</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CJ</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3808,19 +3808,19 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`servises` (en)</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>ASR29W</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3830,24 +3830,24 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`väderingar` (sv)</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3857,24 +3857,24 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>`förforskningsområdet` (sv)</t>
+          <t>`adolscents` (en)</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3884,24 +3884,24 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>`reproduktivhälsaoch` (sv)</t>
+          <t>`indvidual` (en)</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>ASR2CH</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3916,19 +3916,19 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>`perspectiv` (en)</t>
+          <t>`interprofessional` (en)</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>ASR2CJ</t>
+          <t>GSR2ZH</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3943,19 +3943,19 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>`servises` (en)</t>
+          <t>`indvidual` (en)</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2ZH</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>GSR38B</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3965,24 +3965,24 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>`väderingar` (sv)</t>
+          <t>`ukraine` (en)</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>SR3001</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3992,24 +3992,24 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>`adolscents` (en)</t>
+          <t>`hälsodeterminaters` (sv)</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>SR3006</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -4024,19 +4024,19 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>`indvidual` (en)</t>
+          <t>`interferential` (en)</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -4046,24 +4046,24 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>`interprofessional` (en)</t>
+          <t>`hållbarhetsperpektiv` (sv)</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GSR2ZH</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -4073,56 +4073,56 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>`indvidual` (en)</t>
+          <t>`övergripade` (sv)</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2ZH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GSR38B</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>`ukraine` (en)</t>
+          <t>`livsstilförändring` (sv)</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>SR3001</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4132,152 +4132,17 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>`hälsodeterminaters` (sv)</t>
+          <t>`själständigt` (sv)</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>SR3006</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>`interferential` (en)</t>
-        </is>
-      </c>
-      <c r="E138" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="inlineStr">
-        <is>
-          <t>SR3010</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>`hållbarhetsperpektiv` (sv)</t>
-        </is>
-      </c>
-      <c r="E139" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>SR3010</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>`övergripade` (sv)</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>`livsstilförändring` (sv)</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>`själständigt` (sv)</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E142"/>
+  <autoFilter ref="A1:E137"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -4551,16 +4416,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId270"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId271"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A138" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A139" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A140" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A141" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A142" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId282"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update spelling errors and language usage in course plans across multiple analyses
- Revised the "Stavfel och språkbruk" markdown files for IHV, IKS, and ISLL, correcting the number of findings and updating download links for Excel files.
- Adjusted the content in the markdown files to reflect the latest data from the corresponding Excel files, ensuring accuracy in reported spelling errors.
- Updated binary Excel files for Betygsskalor, Bloom-taxonomi, Examinationsformer, Frasningskonsistens, and Introfras across IHV, IKS, and ISLL analyses to reflect the latest changes.
- Ensured consistency in the naming and linking of files for better accessibility.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -985,7 +985,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>IH1001</t>
+          <t>IH1003</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -995,17 +995,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>`rörel-sekompetensen` (sv)</t>
+          <t>`leasure` (en)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>`leasure` (en)</t>
+          <t>`workingform` (en)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1039,7 +1039,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>IH1003</t>
+          <t>IH1004</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1054,19 +1054,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>`workingform` (en)</t>
+          <t>`peda` (en)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1004</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>IH1004</t>
+          <t>IH1024</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1076,24 +1076,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>`peda` (en)</t>
+          <t>`förläsningar` (sv)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1024</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>IH1024</t>
+          <t>IH1114</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>`förläsningar` (sv)</t>
+          <t>`hjäipmedels` (sv)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1114</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>IH1114</t>
+          <t>IH1122</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1130,24 +1130,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>`hjäipmedels` (sv)</t>
+          <t>`hisory` (en)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1114</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1122</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>IH1122</t>
+          <t>IH2002</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1157,29 +1157,29 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`hisory` (en)</t>
+          <t>`rythm` → rhythm (en)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1122</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2002</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>IH2002</t>
+          <t>BKE223</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>KEA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1189,24 +1189,24 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`rythm` → rhythm (en)</t>
+          <t>`stökiometri` (sv)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>IH3007</t>
+          <t>AMC243</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1216,24 +1216,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>`humanbiologi` (en)</t>
+          <t>`naprapath` (en)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>IH3007</t>
+          <t>AMC243</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1243,24 +1243,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`idrottsinriktning` (en)</t>
+          <t>`physiotherpy` (en)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BKE223</t>
+          <t>AMC25W</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>KEA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1270,100 +1270,100 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>`stökiometri` (sv)</t>
+          <t>`ehälsa` (sv)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC25W</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>GNV3GU</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>`naprapath` (en)</t>
+          <t>`inlämingsuppgift` (sv)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>`physiotherpy` (en)</t>
+          <t>`inlämingsuppgift` (sv)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>AMC25W</t>
+          <t>NV1024</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>`ehälsa` (sv)</t>
+          <t>`educationas` (en)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC25W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GNV3GU</t>
+          <t>NV1027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1373,56 +1373,56 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>`inlämingsuppgift` (sv)</t>
+          <t>`adresses` (en)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1027</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>ASA28Q</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>`inlämingsuppgift` (sv)</t>
+          <t>`researcg` (en)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA28Q</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NV1024</t>
+          <t>GSA2AF</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1432,24 +1432,24 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>`educationas` (en)</t>
+          <t>`enablement` (en)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2AF</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>NV1027</t>
+          <t>GSA2BV</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1459,19 +1459,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>`adresses` (en)</t>
+          <t>`enablement` (en)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2BV</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ASA24N</t>
+          <t>GSA2E3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1486,19 +1486,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>`engelskt` (en)</t>
+          <t>`enablement` (en)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA24N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2E3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ASA24N</t>
+          <t>GSA2NC</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1508,24 +1508,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>`namn` (en)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA24N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ASA28Q</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1540,19 +1540,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>`researcg` (en)</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA28Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GSA2AF</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1562,24 +1562,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>`enablement` (en)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2AF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GSA2BV</t>
+          <t>GSA3AS</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1594,19 +1594,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>`enablement` (en)</t>
+          <t>`interorganizational` (en)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2BV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GSA2E3</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1616,24 +1616,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>`enablement` (en)</t>
+          <t>`brukarperspektivinnebär` (sv)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2E3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GSA2NC</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1643,24 +1643,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
+          <t>`frånorganisationsperspektiv` (sv)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GSA2XN</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1670,24 +1670,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>`guidlines` (en)</t>
+          <t>`somarbetslöshet` (sv)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>GSA3DP</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1697,24 +1697,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>SA1037</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>`interorganizational` (en)</t>
+          <t>`övergripandemål` (sv)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1037</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1756,19 +1756,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>`brukarperspektivinnebär` (sv)</t>
+          <t>`skalfrågor` (sv)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1783,19 +1783,19 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>`frånorganisationsperspektiv` (sv)</t>
+          <t>`utvärderbara` (sv)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>SA2020</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1810,24 +1810,24 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>`somarbetslöshet` (sv)</t>
+          <t>`fördjuping` (sv)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GSA3DP</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1837,127 +1837,127 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>`guidlines` (en)</t>
+          <t>`ethhtical` (en)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>SA1037</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>`övergripandemål` (sv)</t>
+          <t>`summarisze` (en)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1037</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR25V</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>`skalfrågor` (sv)</t>
+          <t>`systemacity` (en)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>`utvärderbara` (sv)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>`fördjuping` (sv)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1972,19 +1972,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>`ethhtical` (en)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1999,19 +1999,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>`summarisze` (en)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>ASR25V</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2026,19 +2026,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>`systemacity` (en)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2053,19 +2053,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2080,19 +2080,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`alsoincludes` (en)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`anotherstudent` (en)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2134,19 +2134,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`compilinga` (en)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2161,19 +2161,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`thesisand` (en)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2183,24 +2183,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`föräldrablivande` (sv)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2215,19 +2215,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>`alsoincludes` (en)</t>
+          <t>`beable` (en)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2242,19 +2242,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>`anotherstudent` (en)</t>
+          <t>`processesof` (en)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>`compilinga` (en)</t>
+          <t>`thestudent` (en)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2296,19 +2296,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>`thesisand` (en)</t>
+          <t>`toconduct` (en)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2318,24 +2318,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>`föräldrablivande` (sv)</t>
+          <t>`ofthe` (en)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2350,19 +2350,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>`beable` (en)</t>
+          <t>`postpartumperiod` (en)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>`processesof` (en)</t>
+          <t>`srole` (en)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>`thestudent` (en)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>`toconduct` (en)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2458,19 +2458,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>`ofthe` (en)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2485,19 +2485,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>`postpartumperiod` (en)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2512,19 +2512,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>`srole` (en)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR29W</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2539,19 +2539,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2561,24 +2561,24 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`förforskningsområdet` (sv)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2588,24 +2588,24 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`reproduktivhälsaoch` (sv)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CH</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2620,19 +2620,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`perspectiv` (en)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CJ</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2647,19 +2647,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`servises` (en)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ASR29W</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2669,24 +2669,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`väderingar` (sv)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2696,24 +2696,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>`förforskningsområdet` (sv)</t>
+          <t>`adolscents` (en)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>SR3001</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2728,19 +2728,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>`reproduktivhälsaoch` (sv)</t>
+          <t>`hälsodeterminaters` (sv)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>ASR2CH</t>
+          <t>SR3006</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>`perspectiv` (en)</t>
+          <t>`interferential` (en)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>ASR2CJ</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2777,24 +2777,24 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>`servises` (en)</t>
+          <t>`hållbarhetsperpektiv` (sv)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2809,51 +2809,51 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>`väderingar` (sv)</t>
+          <t>`övergripade` (sv)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>`adolscents` (en)</t>
+          <t>`livsstilförändring` (sv)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>SR3001</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2863,152 +2863,17 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>`hälsodeterminaters` (sv)</t>
+          <t>`själständigt` (sv)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>SR3006</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>`interferential` (en)</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>SR3010</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>`hållbarhetsperpektiv` (sv)</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>SR3010</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>`övergripade` (sv)</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>`livsstilförändring` (sv)</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>`själständigt` (sv)</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E95"/>
+  <autoFilter ref="A1:E90"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -3188,16 +3053,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A90" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A91" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A92" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A93" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A94" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A95" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId188"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update quality notes in course plans for various languages
- Adjusted the number of quality notes in the course plans for Japanese, Chinese, Portuguese, Spanish, and Swedish, reflecting recent reviews and corrections.
- Corrected spelling errors and improved phrasing consistency across multiple course plans.
- Ensured that all course plans maintain a consistent format for quality notes and examination descriptions.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1020,7 +1020,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GIH3D5</t>
+          <t>GIH3F7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1030,30 +1030,30 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>`hälsoin` (sv)</t>
+          <t>`teories` (en)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F7</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GIH3F7</t>
+          <t>GIH3G6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1063,30 +1063,30 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>`teories` (en)</t>
+          <t>`kunskapnivå` (sv)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GIH3G6</t>
+          <t>GIH3JL</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1096,30 +1096,30 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>`kunskapnivå` (sv)</t>
+          <t>`emphasising` (en)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GIH3JL</t>
+          <t>IH1003</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2011-01-26</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>`emphasising` (en)</t>
+          <t>`leasure` (en)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>`leasure` (en)</t>
+          <t>`workingform` (en)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1185,7 +1185,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>IH1003</t>
+          <t>IH1004</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1206,19 +1206,19 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>`workingform` (en)</t>
+          <t>`peda` (en)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1004</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>IH1004</t>
+          <t>IH1024</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1231,27 +1231,31 @@
           <t>2011-01-26</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2012-10-31</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>`peda` (en)</t>
+          <t>`förläsningar` (sv)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1024</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>IH1020</t>
+          <t>IH1114</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1261,14 +1265,10 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2011-01-26</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2012-10-31</t>
-        </is>
-      </c>
+          <t>2015-04-09</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -1276,19 +1276,19 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>`nätb` (sv)</t>
+          <t>`hjäipmedels` (sv)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1114</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>IH1024</t>
+          <t>IH1122</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1298,34 +1298,30 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2011-01-26</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2012-10-31</t>
-        </is>
-      </c>
+          <t>2016-08-26</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>`förläsningar` (sv)</t>
+          <t>`hisory` (en)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1122</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>IH1114</t>
+          <t>IH2002</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1335,7 +1331,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2015-04-09</t>
+          <t>2011-01-26</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1346,128 +1342,128 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>`hjäipmedels` (sv)</t>
+          <t>`rythm` → rhythm (en)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1114</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2002</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>IH1122</t>
+          <t>BKE223</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>KEA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2016-08-26</t>
+          <t>2021-02-17</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>`hisory` (en)</t>
+          <t>`stökiometri` (sv)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH1122</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>IH2002</t>
+          <t>AMC243</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2011-01-26</t>
+          <t>2020-02-20</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>`rythm` → rhythm (en)</t>
+          <t>`naprapath` (en)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BKE223</t>
+          <t>AMC243</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>KEA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2021-02-17</t>
+          <t>2020-02-20</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>`stökiometri` (sv)</t>
+          <t>`physiotherpy` (en)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>GNV3GU</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1478,65 +1474,69 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>`metodövnin` (sv)</t>
+          <t>`inlämingsuppgift` (sv)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>`naprapath` (en)</t>
+          <t>`inlämingsuppgift` (sv)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>NV1024</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>2012-10-11</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2014-02-12</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1544,231 +1544,231 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>`physiotherpy` (en)</t>
+          <t>`educationas` (en)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1024</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>AMC29Y</t>
+          <t>NV1027</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2023-12-05</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>2013-03-15</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2014-02-12</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>`läkem` (sv)</t>
+          <t>`adresses` (en)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1027</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AMC2BG</t>
+          <t>ASA28Q</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>`läkem` (sv)</t>
+          <t>`researcg` (en)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2BG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA28Q</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>MC1077</t>
+          <t>GSA2NC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2015-02-12</t>
+          <t>2021-03-09</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>`läkemedelsh` (sv)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MC1077</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>MC1079</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2015-06-11</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2015-08-18</t>
-        </is>
-      </c>
+          <t>2022-09-08</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>`läkemed` (sv)</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MC1079</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>MC3027</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2017-03-13</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>`läkem` (sv)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MC3027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GNV3GU</t>
+          <t>GSA3AS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2024-03-04</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>`inlämingsuppgift` (sv)</t>
+          <t>`interorganizational` (en)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2024-12-10</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1779,93 +1779,85 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>`inlämingsuppgift` (sv)</t>
+          <t>`brukarperspektivinnebär` (sv)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>NV1024</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2012-10-11</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2014-02-12</t>
-        </is>
-      </c>
+          <t>2024-12-10</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>`educationas` (en)</t>
+          <t>`frånorganisationsperspektiv` (sv)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>NV1027</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2013-03-15</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2014-02-12</t>
-        </is>
-      </c>
+          <t>2024-12-10</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>`adresses` (en)</t>
+          <t>`somarbetslöshet` (sv)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NV1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ASA28Q</t>
+          <t>GSA3DP</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1875,7 +1867,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2024-12-10</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1886,19 +1878,19 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>`researcg` (en)</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA28Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GSA2AF</t>
+          <t>SA1037</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1908,14 +1900,10 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2019-08-29</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2023-09-13</t>
-        </is>
-      </c>
+          <t>2015-03-11</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -1923,19 +1911,19 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>`såd` (sv)</t>
+          <t>`övergripandemål` (sv)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2AF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1037</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GSA2NC</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1945,30 +1933,30 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2021-03-09</t>
+          <t>2016-05-20</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>`credits` — ……7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits… | &gt; |…</t>
+          <t>`skalfrågor` (sv)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GSA2XN</t>
+          <t>SA1040</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1978,30 +1966,30 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
+          <t>2016-05-20</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>`guidlines` (en)</t>
+          <t>`utvärderbara` (sv)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>SA2020</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2011,40 +1999,40 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2014-12-23</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>`credits` — ……7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits… | &lt;!-…</t>
+          <t>`fördjuping` (sv)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2018-12-06</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -2055,128 +2043,132 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>`interorganizational` (en)</t>
+          <t>`ethhtical` (en)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2018-12-06</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>`brukarperspektivinnebär` (sv)</t>
+          <t>`summarisze` (en)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>ASR25V</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
+          <t>2020-06-17</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2020-06-25</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>`frånorganisationsperspektiv` (sv)</t>
+          <t>`systemacity` (en)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2022-06-16</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>`somarbetslöshet` (sv)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GSA3DP</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2022-06-16</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -2187,250 +2179,250 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>`guidlines` (en)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>SA1037</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2015-03-11</t>
+          <t>2022-06-16</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>`övergripandemål` (sv)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1037</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2016-05-20</t>
+          <t>2022-06-16</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>`skalfrågor` (sv)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2016-05-20</t>
+          <t>2022-06-16</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>`utvärderbara` (sv)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2014-12-23</t>
+          <t>2022-06-16</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>`fördjuping` (sv)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2014-12-23</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>`såd` (sv)</t>
+          <t>`alsoincludes` (en)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2014-12-23</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>`utvärderi` (sv)</t>
+          <t>`anotherstudent` (en)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>SA3008</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2016-09-08</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>`såd` (sv)</t>
+          <t>`compilinga` (en)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA3008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2440,7 +2432,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2018-12-06</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -2451,19 +2443,19 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>`ethhtical` (en)</t>
+          <t>`thesisand` (en)</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2473,30 +2465,30 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2018-12-06</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>`summarisze` (en)</t>
+          <t>`föräldrablivande` (sv)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ASR25V</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2506,14 +2498,10 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2020-06-17</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2020-06-25</t>
-        </is>
-      </c>
+          <t>2023-10-03</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2521,19 +2509,19 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>`systemacity` (en)</t>
+          <t>`beable` (en)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2543,7 +2531,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -2554,19 +2542,19 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`processesof` (en)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2576,7 +2564,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -2587,19 +2575,19 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`thestudent` (en)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2609,7 +2597,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -2620,19 +2608,19 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`toconduct` (en)</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2642,7 +2630,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -2653,19 +2641,19 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`ofthe` (en)</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2675,7 +2663,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -2686,19 +2674,19 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`postpartumperiod` (en)</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2708,7 +2696,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -2719,19 +2707,19 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`srole` (en)</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2752,19 +2740,19 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>`alsoincludes` (en)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2785,19 +2773,19 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>`anotherstudent` (en)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2818,19 +2806,19 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>`compilinga` (en)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2851,19 +2839,19 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>`thesisand` (en)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2879,24 +2867,24 @@
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>`föräldrablivande` (sv)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29W</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2917,19 +2905,19 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>`beable` (en)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2939,30 +2927,30 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>`processesof` (en)</t>
+          <t>`förforskningsområdet` (sv)</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2972,30 +2960,30 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>`thestudent` (en)</t>
+          <t>`reproduktivhälsaoch` (sv)</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR2CH</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3005,7 +2993,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -3016,19 +3004,19 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>`toconduct` (en)</t>
+          <t>`perspectiv` (en)</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR2CJ</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3038,7 +3026,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -3049,19 +3037,19 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>`ofthe` (en)</t>
+          <t>`servises` (en)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR2CR</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3071,7 +3059,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -3082,19 +3070,19 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>`postpartumperiod` (en)</t>
+          <t>`andother` (en)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR2CR</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3104,7 +3092,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -3115,19 +3103,19 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>`srole` (en)</t>
+          <t>`carewithin` (en)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CR</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3137,7 +3125,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -3148,19 +3136,19 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`postpartumperiod` (en)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3170,7 +3158,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -3181,19 +3169,19 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`beable` (en)</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CS</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3203,30 +3191,34 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
+          <t>2019-06-19</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>2021-02-19</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`väderingar` (sv)</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3236,10 +3228,14 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
+          <t>2019-06-19</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2021-02-19</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -3247,19 +3243,19 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`adolscents` (en)</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>SR3001</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3269,30 +3265,30 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2016-10-05</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`hälsodeterminaters` (sv)</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>ASR29W</t>
+          <t>SR3006</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3302,7 +3298,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2016-10-05</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
@@ -3313,19 +3309,19 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`interferential` (en)</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3335,10 +3331,14 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
+          <t>2016-10-12</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2017-10-05</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -3346,19 +3346,19 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>`förforskningsområdet` (sv)</t>
+          <t>`hållbarhetsperpektiv` (sv)</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3368,10 +3368,14 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
+          <t>2016-10-12</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>2017-10-05</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -3379,234 +3383,242 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>`reproduktivhälsaoch` (sv)</t>
+          <t>`övergripade` (sv)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ASR2CH</t>
+          <t>VBSKA</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2019-09-10</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>`perspectiv` (en)</t>
+          <t>`europarådets` (sv)</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ASR2CJ</t>
+          <t>VBSKA</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2019-09-10</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>`servises` (en)</t>
+          <t>`postpartumvård` (sv)</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ASR2CR</t>
+          <t>VBSKA</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2019-09-10</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>`andother` (en)</t>
+          <t>`ternström` (sv)</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ASR2CR</t>
+          <t>VDSSA</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr"/>
+          <t>2018-12-04</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2022-06-22</t>
+        </is>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>`carewithin` (en)</t>
+          <t>`hälso` (sv)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ASR2CR</t>
+          <t>VDSSA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
+          <t>2018-12-04</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2022-06-22</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>`postpartumperiod` (en)</t>
+          <t>`levnadsvaneförändring` (sv)</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ASR2CS</t>
+          <t>VDSSA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
+          <t>2018-12-04</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>2022-06-22</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>`beable` (en)</t>
+          <t>`levnadsvaneförändringar` (sv)</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CS</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>VSADA</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>2021-02-19</t>
-        </is>
-      </c>
+          <t>2023-01-09</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -3614,66 +3626,62 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>`väderingar` (sv)</t>
+          <t>`engström` (sv)</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>VSADA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>2021-02-19</t>
-        </is>
-      </c>
+          <t>2023-01-09</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>`adolscents` (en)</t>
+          <t>`ätandeproblem` (sv)</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>SR3001</t>
+          <t>VSJPG</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2016-10-05</t>
+          <t>2023-11-07</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
@@ -3684,29 +3692,29 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>`hälsodeterminaters` (sv)</t>
+          <t>`engström` (sv)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSJPG</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>SR3005</t>
+          <t>VSOPG</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2016-10-05</t>
+          <t>2021-02-04</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -3717,67 +3725,71 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>`ansvarsområd` (sv)</t>
+          <t>`hälso` (sv)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3005</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSOPG</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>SR3006</t>
+          <t>VSSKG</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2016-10-05</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr"/>
+          <t>2018-12-04</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>2020-12-17</t>
+        </is>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>`interferential` (en)</t>
+          <t>`engström` (sv)</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>SR3009</t>
+          <t>VSSKG</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2016-10-12</t>
+          <t>2018-12-04</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2017-10-05</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -3787,34 +3799,34 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>`hälsotill` (sv)</t>
+          <t>`hälso` (sv)</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>SR3009</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2016-10-12</t>
+          <t>2010-06-01</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2017-10-05</t>
+          <t>2010-10-18</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3824,34 +3836,34 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>`mänsk` (sv)</t>
+          <t>`livsstilförändring` (sv)</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>SR3010</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2016-10-12</t>
+          <t>2010-06-01</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2017-10-05</t>
+          <t>2010-10-18</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -3861,34 +3873,34 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>`hållbarhetsperpektiv` (sv)</t>
+          <t>`själständigt` (sv)</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>SR3010</t>
+          <t>FHV0002</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅRDVETS</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2016-10-12</t>
+          <t>2018-03-28</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2017-10-05</t>
+          <t>2022-09-28</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -3898,725 +3910,91 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>`övergripade` (sv)</t>
+          <t>`valitetsbedömning` (sv)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>VBSKA</t>
+          <t>FHV0002</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Utbildningsplaner</t>
+          <t>VÅRDVETS</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2019-09-10</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
+          <t>2018-03-28</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2022-09-28</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>`europarådets` (sv)</t>
+          <t>`cerqual` (en)</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>VBSKA</t>
+          <t>FVV222H</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Utbildningsplaner</t>
+          <t>VÅRDVETS</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2019-09-10</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr"/>
+          <t>2022-04-28</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>2023-01-19</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>`postpartumvård` (sv)</t>
+          <t>`isues` (en)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>VBSKA</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>2019-09-10</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>`ternström` (sv)</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>VDSSA</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>2022-06-22</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>VDSSA</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>2022-06-22</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>`levnadsvaneförändring` (sv)</t>
-        </is>
-      </c>
-      <c r="G108" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>VDSSA</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>2022-06-22</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>`levnadsvaneförändringar` (sv)</t>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>VSADA</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>2023-01-09</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>VSADA</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>2023-01-09</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>`ätandeproblem` (sv)</t>
-        </is>
-      </c>
-      <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>VSJPG</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>2023-11-07</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G112" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSJPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>VSOPG</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>2021-02-04</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr"/>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G113" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSOPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>VSSKG</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>VSSKG</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G115" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>AVV26K</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>2021-02-24</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>2021-03-02</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>`inlä` (sv)</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV26K</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>VV2002</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>2009-09-01</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>2012-03-05</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>`äldreomso` (sv)</t>
-        </is>
-      </c>
-      <c r="G117" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV2002</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>2010-06-01</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>2010-10-18</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>`livsstilförändring` (sv)</t>
-        </is>
-      </c>
-      <c r="G118" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>2010-06-01</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>2010-10-18</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>`själständigt` (sv)</t>
-        </is>
-      </c>
-      <c r="G119" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>FHV0001</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>2018-01-25</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>`redogöre` (sv)</t>
-        </is>
-      </c>
-      <c r="G120" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>FHV0002</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>2018-03-28</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>2022-09-28</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>`valitetsbedömning` (sv)</t>
-        </is>
-      </c>
-      <c r="G121" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>FHV0002</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>2018-03-28</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>2022-09-28</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>`cerqual` (en)</t>
-        </is>
-      </c>
-      <c r="G122" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t>FVV222H</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>2022-04-28</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>2023-01-19</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>`isues` (en)</t>
-        </is>
-      </c>
-      <c r="G123" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FVV222H</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G123"/>
+  <autoFilter ref="A1:G105"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -4826,42 +4204,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId207"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A113" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A114" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A120" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A121" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A122" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A123" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId244"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix quality notes in course plans and update related documentation
- Updated the number of quality notes in multiple course plans to reflect recent changes.
- Corrected spelling errors and language usage in course descriptions.
- Adjusted the formatting of examination forms and learning outcomes for consistency.
- Removed outdated references to courses that have been discontinued.
- Updated links and download information in analysis documents.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -517,83 +517,83 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BKE223</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KEA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2021-02-17</t>
+          <t>2022-09-08</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>`stökiometri` (sv)</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BKE223</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AMC243</t>
+          <t>SA2020</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
+          <t>2014-12-23</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>`naprapath` (en)</t>
+          <t>`fördjuping` (sv)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC243</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GSA2XN</t>
+          <t>ASR22N</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
+          <t>2018-12-06</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -604,29 +604,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>`guidlines` (en)</t>
+          <t>`ethtical` (en)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -637,118 +637,118 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>`interorganizational` (en)</t>
+          <t>`alsoincludes` (en)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2016-05-20</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>`skalfrågor` (sv)</t>
+          <t>`anotherstudent` (en)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SA1040</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2016-05-20</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>`utvärderbara` (sv)</t>
+          <t>`compilinga` (en)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2014-12-23</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>`fördjuping` (sv)</t>
+          <t>`thesisand` (en)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ASR22N</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2018-12-06</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -769,19 +769,19 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>`ethtical` (en)</t>
+          <t>`beable` (en)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ASR25V</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -791,14 +791,10 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2020-06-17</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2020-06-25</t>
-        </is>
-      </c>
+          <t>2023-10-03</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -806,19 +802,19 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>`systematicity` (en)</t>
+          <t>`processesof` (en)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -839,19 +835,19 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>`alsoincludes` (en)</t>
+          <t>`thestudent` (en)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -872,19 +868,19 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>`anotherstudent` (en)</t>
+          <t>`toconduct` (en)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -905,19 +901,19 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>`compilinga` (en)</t>
+          <t>`ofthe` (en)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -938,19 +934,19 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>`thesisand` (en)</t>
+          <t>`postpartumperiod` (en)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -966,24 +962,24 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>`föräldrablivande` (sv)</t>
+          <t>`srole` (en)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1004,19 +1000,19 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>`beable` (en)</t>
+          <t>`carrid` (en)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1037,19 +1033,19 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>`processesof` (en)</t>
+          <t>`focsing` (en)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1070,19 +1066,19 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>`thestudent` (en)</t>
+          <t>`havng` (en)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1103,19 +1099,19 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>`toconduct` (en)</t>
+          <t>`situaion` (en)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1136,19 +1132,19 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>`ofthe` (en)</t>
+          <t>`traied` (en)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29W</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1169,19 +1165,19 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>`postpartumperiod` (en)</t>
+          <t>`ofa` (en)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1191,30 +1187,30 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>`srole` (en)</t>
+          <t>`förforskningsområdet` (sv)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CF</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1224,30 +1220,30 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>`carrid` (en)</t>
+          <t>`reproduktivhälsaoch` (sv)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CH</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1257,7 +1253,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1268,19 +1264,19 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>`focsing` (en)</t>
+          <t>`perspectiv` (en)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CJ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1290,7 +1286,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1301,19 +1297,19 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>`havng` (en)</t>
+          <t>`servises` (en)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CR</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1323,7 +1319,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1334,19 +1330,19 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>`situaion` (en)</t>
+          <t>`andother` (en)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR2CR</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1356,7 +1352,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1367,19 +1363,19 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>`traied` (en)</t>
+          <t>`carewithin` (en)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ASR29W</t>
+          <t>ASR2CR</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1389,7 +1385,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1400,19 +1396,19 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>`ofa` (en)</t>
+          <t>`postpartumperiod` (en)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>ASR2CS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1422,30 +1418,30 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>`förforskningsområdet` (sv)</t>
+          <t>`beable` (en)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ASR2CF</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1455,10 +1451,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>2019-06-19</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2021-02-19</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -1466,19 +1466,19 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>`reproduktivhälsaoch` (sv)</t>
+          <t>`väderingar` (sv)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ASR2CH</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1488,10 +1488,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>2019-06-19</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2021-02-19</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1499,19 +1503,19 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>`perspectiv` (en)</t>
+          <t>`adolscents` (en)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ASR2CJ</t>
+          <t>SR3001</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1521,30 +1525,30 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2016-10-05</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>`servises` (en)</t>
+          <t>`hälsodeterminaters` (sv)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ASR2CR</t>
+          <t>SR3006</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1554,7 +1558,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2016-10-05</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1565,19 +1569,19 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>`andother` (en)</t>
+          <t>`interferential` (en)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ASR2CR</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1587,30 +1591,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>2016-10-12</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2017-10-05</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>`carewithin` (en)</t>
+          <t>`hållbarhetsperpektiv` (sv)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ASR2CR</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1620,80 +1628,80 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>2016-10-12</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2017-10-05</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>`postpartumperiod` (en)</t>
+          <t>`övergripade` (sv)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ASR2CS</t>
+          <t>VBSKA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2019-09-10</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>`beable` (en)</t>
+          <t>`europarådets` (sv)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CS</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>VBSKA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2021-02-19</t>
-        </is>
-      </c>
+          <t>2019-09-10</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -1701,69 +1709,69 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>`väderingar` (sv)</t>
+          <t>`postpartumvård` (sv)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>VBSKA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2021-02-19</t>
-        </is>
-      </c>
+          <t>2019-09-10</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>`adolscents` (en)</t>
+          <t>`ternström` (sv)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SR3001</t>
+          <t>VDSSA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2016-10-05</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>2018-12-04</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2022-06-22</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -1771,67 +1779,71 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>`hälsodeterminaters` (sv)</t>
+          <t>`hälso` (sv)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SR3006</t>
+          <t>VDSSA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2016-10-05</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>2018-12-04</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2022-06-22</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>`interferential` (en)</t>
+          <t>`levnadsvaneförändring` (sv)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3006</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SR3010</t>
+          <t>VDSSA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2016-10-12</t>
+          <t>2018-12-04</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2017-10-05</t>
+          <t>2022-06-22</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1841,36 +1853,32 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>`hållbarhetsperpektiv` (sv)</t>
+          <t>`levnadsvaneförändringar` (sv)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>SR3010</t>
+          <t>VSADA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>Utbildningsplaner</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2016-10-12</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2017-10-05</t>
-        </is>
-      </c>
+          <t>2023-01-09</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -1878,19 +1886,19 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>`övergripade` (sv)</t>
+          <t>`engström` (sv)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>VBSKA</t>
+          <t>VSADA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1900,7 +1908,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2019-09-10</t>
+          <t>2023-01-09</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1911,19 +1919,19 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>`europarådets` (sv)</t>
+          <t>`ätandeproblem` (sv)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>VBSKA</t>
+          <t>VSJPG</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1933,7 +1941,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2019-09-10</t>
+          <t>2023-11-07</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1944,19 +1952,19 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>`postpartumvård` (sv)</t>
+          <t>`engström` (sv)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSJPG</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>VBSKA</t>
+          <t>VSOPG</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1966,7 +1974,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2019-09-10</t>
+          <t>2021-02-04</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1977,19 +1985,19 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>`ternström` (sv)</t>
+          <t>`hälso` (sv)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSOPG</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>VDSSA</t>
+          <t>VSSKG</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2004,7 +2012,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2022-06-22</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2014,19 +2022,19 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>`hälso` (sv)</t>
+          <t>`engström` (sv)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>VDSSA</t>
+          <t>VSSKG</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2041,7 +2049,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2022-06-22</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2051,34 +2059,34 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>`levnadsvaneförändring` (sv)</t>
+          <t>`hälso` (sv)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>VDSSA</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Utbildningsplaner</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2018-12-04</t>
+          <t>2010-06-01</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2022-06-22</t>
+          <t>2010-10-18</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2088,32 +2096,36 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>`levnadsvaneförändringar` (sv)</t>
+          <t>`livsstilförändring` (sv)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>VSADA</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Utbildningsplaner</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2023-01-09</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
+          <t>2010-06-01</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2010-10-18</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -2121,32 +2133,36 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>`engström` (sv)</t>
+          <t>`själständigt` (sv)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>VSADA</t>
+          <t>FHV0002</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Utbildningsplaner</t>
+          <t>VÅRDVETS</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2023-01-09</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
+          <t>2018-03-28</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2022-09-28</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -2154,342 +2170,54 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>`ätandeproblem` (sv)</t>
+          <t>`valitetsbedömning` (sv)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>VSJPG</t>
+          <t>FVV222H</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Utbildningsplaner</t>
+          <t>VÅRDVETS</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
+          <t>2022-04-28</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2023-01-19</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>`engström` (sv)</t>
+          <t>`isues` (en)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSJPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>VSOPG</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>2021-02-04</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSOPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>VSSKG</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>VSSKG</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>2010-06-01</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2010-10-18</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>`livsstilförändring` (sv)</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>VV3011</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>VÅE</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>2010-06-01</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2010-10-18</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>`själständigt` (sv)</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>FHV0002</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>2018-03-28</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>2022-09-28</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>`valitetsbedömning` (sv)</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>FHV0002</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>2018-03-28</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>2022-09-28</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>`cerqual` (en)</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>FVV222H</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>VÅRDVETS</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>2022-04-28</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>2023-01-19</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>`isues` (en)</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FVV222H</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G60"/>
+  <autoFilter ref="A1:G52"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -2593,22 +2321,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId118"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new valid terms and update various Excel reports
- Updated `checks_common.py` to include new valid terms related to education and health.
- Modified multiple Excel files across different university departments (IIT, IHV, IKS, ISLL) to reflect changes in grading reports, examination formats, and other analyses.
- Adjusted markdown files to update links and correct spelling errors in course descriptions and references.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -650,424 +650,8 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>VBSKA</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2019-09-10</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>`europarådets` (sv)</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>VBSKA</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2019-09-10</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>`postpartumvård` (sv)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>VBSKA</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2019-09-10</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>`ternström` (sv)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>VDSSA</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2022-06-22</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>VDSSA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2022-06-22</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>`levnadsvaneförändring` (sv)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>VDSSA</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2022-06-22</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>`levnadsvaneförändringar` (sv)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VDSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>VSADA</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2023-01-09</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>VSADA</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2023-01-09</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>`ätandeproblem` (sv)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>VSJPG</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2023-11-07</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSJPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>VSOPG</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2021-02-04</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSOPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>VSSKG</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>`engström` (sv)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>VSSKG</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2018-12-04</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>`hälso` (sv)</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSSKG</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G18"/>
+  <autoFilter ref="A1:G6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -1079,30 +663,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans for Ljud- och musikproduktion: mark courses as "nedlagd" and add draft status. Adjusted course listings and removed inactive courses from the main section. Updated various analysis Excel files for ISLL.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -484,17 +484,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-09-08</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -505,164 +505,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>`collaboratation` (en)</t>
+          <t>`guidlines` (en)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>GSA2XN</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SAA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2022-09-08</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>`guidlines` (en)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>SA2020</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SAA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2014-12-23</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>`fördjuping` (sv)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>ASR22N</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2018-12-06</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>`ethtical` (en)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR22N</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>GSR2A5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SRP</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2019-06-19</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2021-02-19</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>`adolscents` (en)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:G2"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>